<commit_message>
added name id email and tut no.
</commit_message>
<xml_diff>
--- a/PopEyez requirements.xlsx
+++ b/PopEyez requirements.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tonyj\OneDrive\Desktop\projects\PopEyez\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d82daf92372a5c5a/Desktop/projects/PopEyez/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69A0B25-CFAB-44AE-B65B-BA50535A5F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{E69A0B25-CFAB-44AE-B65B-BA50535A5F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2669907C-96B3-48BF-BE23-345705B145F3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3380" yWindow="3380" windowWidth="19200" windowHeight="9970" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team Info" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="215">
   <si>
     <t>Team Name</t>
   </si>
@@ -670,6 +670,12 @@
   </si>
   <si>
     <t>I can approve payment and update my budget.</t>
+  </si>
+  <si>
+    <t>Tony John Safwat Gendy</t>
+  </si>
+  <si>
+    <t>tony.gendy@student.giu-berlin.de</t>
   </si>
 </sst>
 </file>
@@ -997,7 +1003,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1147,6 +1153,12 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1156,12 +1168,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1366,38 +1373,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
     </row>
     <row r="2" spans="1:4" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="68"/>
-      <c r="B2" s="68"/>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
+      <c r="A2" s="70"/>
+      <c r="B2" s="70"/>
+      <c r="C2" s="70"/>
+      <c r="D2" s="70"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="68"/>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
+      <c r="A3" s="70"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
     </row>
     <row r="4" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="68"/>
-      <c r="B4" s="68"/>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
+      <c r="A4" s="70"/>
+      <c r="B4" s="70"/>
+      <c r="C4" s="70"/>
+      <c r="D4" s="70"/>
     </row>
     <row r="5" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69"/>
-      <c r="D5" s="69"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="71"/>
+      <c r="D5" s="71"/>
     </row>
     <row r="6" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
@@ -1470,10 +1477,18 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="13" x14ac:dyDescent="0.3">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
+      <c r="A11" s="11" t="s">
+        <v>213</v>
+      </c>
+      <c r="B11" s="12">
+        <v>22001215</v>
+      </c>
+      <c r="C11" s="72" t="s">
+        <v>214</v>
+      </c>
+      <c r="D11" s="12">
+        <v>2</v>
+      </c>
     </row>
     <row r="12" spans="1:4" ht="13" x14ac:dyDescent="0.3">
       <c r="A12" s="13"/>
@@ -1489,6 +1504,7 @@
     <hyperlink ref="C8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="C9" r:id="rId3" xr:uid="{693CED25-6D74-40F0-ABD4-E90771578C28}"/>
     <hyperlink ref="C10" r:id="rId4" xr:uid="{55D1C066-3F5F-4DDC-ABBD-5BC351D74261}"/>
+    <hyperlink ref="C11" r:id="rId5" xr:uid="{3FF22B8B-602F-4D46-823E-CD5FCEB28965}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1509,29 +1525,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="70" t="s">
+      <c r="B1" s="67" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="70" t="s">
+      <c r="C1" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="71" t="s">
+      <c r="D1" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="70" t="s">
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="67" t="s">
         <v>14</v>
       </c>
       <c r="J1" s="14"/>
     </row>
     <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="70"/>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
+      <c r="A2" s="67"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
       <c r="D2" s="15" t="s">
         <v>15</v>
       </c>
@@ -1541,7 +1557,7 @@
       <c r="F2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="70"/>
+      <c r="G2" s="67"/>
       <c r="J2" s="16"/>
     </row>
     <row r="3" spans="1:25" ht="12.5" x14ac:dyDescent="0.25">

</xml_diff>